<commit_message>
docs(dictionary): update fields and values (Google, thresholds, home types)
</commit_message>
<xml_diff>
--- a/Base de datos/Diccionario de Datos.xlsx
+++ b/Base de datos/Diccionario de Datos.xlsx
@@ -30,6 +30,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alert" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recommendation" sheetId="26" state="visible" r:id="rId26"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notification" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NotificationPreference" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PushSubscription" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39,7 +41,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Aptos Narrow"/>
       <color theme="1"/>
@@ -68,6 +70,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -156,7 +162,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -196,6 +202,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -577,11 +584,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="0" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
+      <c r="A7" s="0" t="n"/>
       <c r="B7" s="0" t="inlineStr">
         <is>
           <t>last_name</t>
@@ -599,7 +602,7 @@
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>Apellidos de la persona</t>
+          <t>Apellidos de la persona (NULL en cuentas de Google sin apellido)</t>
         </is>
       </c>
     </row>
@@ -1658,7 +1661,7 @@
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t>Nombre del tipo de hogar</t>
+          <t>Nombre del tipo de hogar (valores: house, apartment, studio, country_house, cabin, other)</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="8" min="1" max="1"/>
@@ -2161,15 +2164,42 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="0" t="inlineStr">
-        <is>
-          <t>Relaciones:</t>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>limit_period</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>ENUM</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>DAILY, MONTHLY</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t>Periodo del límite configurado (diario o mensual)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>Relaciones:</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>HomeThresholds 1:1 Home</t>
         </is>
@@ -2511,7 +2541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="8" min="1" max="1"/>
@@ -2790,64 +2820,88 @@
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t>VARCHAR</t>
-        </is>
-      </c>
-      <c r="D14" s="0" t="inlineStr">
+          <t>MEDIUMTEXT</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="n"/>
+      <c r="E14" s="0" t="inlineStr">
+        <is>
+          <t>Imagen de perfil del usuario como data URL (MEDIUMTEXT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>UNIQUE</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>google_subject</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>VARCHAR</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>255</t>
         </is>
       </c>
-      <c r="E14" s="0" t="inlineStr">
-        <is>
-          <t>Ruta o URL de la imagen de perfil de la cuenta</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="0" t="inlineStr">
-        <is>
-          <t>Relaciones:</t>
-        </is>
-      </c>
-    </row>
+      <c r="E15" s="0" t="inlineStr">
+        <is>
+          <t>Identificador (sub) de la cuenta de Google; NULL en cuentas con contraseña</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>User 1:1 Person</t>
+          <t>Relaciones:</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>User 1:1 UserConfiguration</t>
+          <t>User 1:1 Person</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>User 1:N PasswordResetToken</t>
+          <t>User 1:1 UserConfiguration</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>User 1:N UserSession</t>
+          <t>User 1:N PasswordResetToken</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>User 1:N UserSystemRole</t>
+          <t>User 1:N UserSession</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>User 1:N UserSystemRole</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
         <is>
           <t>User 1:N AuditLog</t>
         </is>
@@ -3347,13 +3401,13 @@
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>TIMESTAMP</t>
+          <t>TIMESTAMP(6)</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr"/>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t>Última fecha de conexión</t>
+          <t>Última fecha de conexión (precisión de microsegundos)</t>
         </is>
       </c>
     </row>
@@ -3999,7 +4053,7 @@
     <row r="2" ht="32" customHeight="1" s="8">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t>Descripción: Registra alertas de umbral y conectividad.</t>
+          <t>Descripción: Registra alertas de umbral, conectividad, eventos de dispositivo y límite de consumo.</t>
         </is>
       </c>
     </row>
@@ -4280,7 +4334,7 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>Alert N:1 Measurement</t>
+          <t>type: THRESHOLD, CONNECTIVITY, DEVICE, LIMIT</t>
         </is>
       </c>
     </row>
@@ -4299,7 +4353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="8" min="1" max="1"/>
@@ -4485,7 +4539,7 @@
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>type</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -4496,7 +4550,7 @@
       <c r="D10" s="0" t="inlineStr"/>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>Estado de lectura</t>
+          <t>Tipo de recomendación</t>
         </is>
       </c>
     </row>
@@ -4508,7 +4562,7 @@
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>status</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -4519,7 +4573,7 @@
       <c r="D11" s="0" t="inlineStr"/>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t>Tipo de recomendación</t>
+          <t>Estado de lectura</t>
         </is>
       </c>
     </row>
@@ -4541,6 +4595,20 @@
       <c r="A15" s="0" t="inlineStr">
         <is>
           <t>Recommendation N:1 Device</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>type: SAVING, PEAK_HOURS, HIGH_CONSUMPTION, HISTORICAL_COMPARISON, THRESHOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>status: READ, UNREAD</t>
         </is>
       </c>
     </row>
@@ -4563,318 +4631,663 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="0" t="inlineStr">
         <is>
           <t>Notification</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>Descripción: Registro de entrega de un mensaje al usuario. Alert y Recommendation son eventos; Notification registra si el mensaje fue entregado, por qué canal y su estado de lectura.</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>Clave</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>Campo</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>Tipo de Dato</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>Tamaño</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>id_notification</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>VARCHAR</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>VARCHAR</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
         <is>
           <t>user_id</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>VARCHAR</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>VARCHAR</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr"/>
+      <c r="B7" s="0" t="inlineStr">
         <is>
           <t>home_id</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>VARCHAR</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>VARCHAR</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
         <is>
           <t>channel</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>ENUM</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>EMAIL,PUSH</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>source_type</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>ENUM</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>ALERT,RECOMMENDATION</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr"/>
+      <c r="B10" s="0" t="inlineStr">
         <is>
           <t>source_id</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>VARCHAR</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>VARCHAR</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
         <is>
           <t>message_key</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>VARCHAR</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>VARCHAR</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
         <is>
           <t>delivery_status</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>ENUM</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>PENDING,SENT,FAILED</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr"/>
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>sent_at</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr"/>
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>read_at</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr"/>
+      <c r="B15" s="0" t="inlineStr">
         <is>
           <t>failure_reason</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>VARCHAR</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>VARCHAR</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr"/>
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr"/>
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>updated_at</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr"/>
+      <c r="B18" s="0" t="inlineStr">
         <is>
           <t>deleted_at</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
         <is>
           <t>Relaciones:</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
         <is>
           <t>Notification N:1 User (referencia aplicación)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="0" t="inlineStr">
         <is>
           <t>Notification N:1 Home (referencia aplicación)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>Notification referencia Alert/Recommendation por (source_type, source_id)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>NotificationPreference</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>Descripción: Preferencias de canal de notificación por usuario. Sin fila se aplican los valores por defecto (ambos activos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Clave</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>Campo</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>Tipo de Dato</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>Tamaño</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>user_id</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>VARCHAR</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>Usuario propietario de la preferencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>email_enabled</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr"/>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>Notificaciones por correo habilitadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>push_enabled</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr"/>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>Notificaciones push habilitadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Relaciones:</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NotificationPreference N:1 User (referencia aplicación)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>PushSubscription</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>Descripción: Navegadores suscritos a Web Push. endpoint identifica la instalación; p256dh y auth cifran el payload (RFC 8291).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Clave</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>Campo</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>Tipo de Dato</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>Tamaño</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>id_push_subscription</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>VARCHAR</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>Identificador de la suscripción</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>user_id</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>VARCHAR</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>Usuario suscrito</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>UNIQUE / NOT NULL</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>endpoint</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>VARCHAR</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>Endpoint del navegador</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>p256dh</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>VARCHAR</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>Clave pública del navegador</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>auth</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>VARCHAR</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>Secreto de autenticación</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Relaciones:</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>PushSubscription N:1 User</t>
         </is>
       </c>
     </row>
@@ -5138,7 +5551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="8" min="1" max="1"/>
@@ -5251,7 +5664,7 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>reset_token</t>
+          <t>reset_token_hash</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -5261,12 +5674,12 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>64</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>Token de recuperación</t>
+          <t>Hash del token de recuperación</t>
         </is>
       </c>
     </row>
@@ -5301,30 +5714,53 @@
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
+          <t>attempts</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="n"/>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>Intentos fallidos de canje</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
           <t>expiration_at</t>
         </is>
       </c>
-      <c r="C9" s="0" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
       </c>
-      <c r="D9" s="0" t="inlineStr"/>
-      <c r="E9" s="0" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr"/>
+      <c r="E10" s="0" t="inlineStr">
         <is>
           <t>Fecha de expiración</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="0" t="inlineStr">
-        <is>
-          <t>Relaciones:</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>Relaciones:</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>PasswordResetToken N:1 User</t>
         </is>

</xml_diff>